<commit_message>
Expand Speedgoat video URLs sheet with YouTube and MathWorks videos
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012aPLXV7VPSpNbmEkkkyZuV
</commit_message>
<xml_diff>
--- a/speedgoat_video_urls.xlsx
+++ b/speedgoat_video_urls.xlsx
@@ -7,9 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Video URLs" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Video pages (no 'video' in URL)" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Notes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Speedgoat.com video URLs" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="YouTube videos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="MathWorks-hosted videos" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Video pages (no 'video' in URL)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Notes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -453,10 +455,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="72" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="1" max="1"/>
     <col width="115" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -468,7 +470,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Speedgoat URL</t>
+          <t>URL</t>
         </is>
       </c>
     </row>
@@ -592,15 +594,321 @@
         </is>
       </c>
     </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="80" customWidth="1" min="1" max="1"/>
+    <col width="115" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Speedgoat YouTube channel (@SpeedgoatRT) - ALL videos live here</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@SpeedgoatRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Speedgoat YouTube channel - videos tab</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/c/SpeedgoatCh/videos</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Speedgoat YouTube channel (channel ID)</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/channel/UCmVuPugCbMDOjocC529tdRg</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>How to perform real-time simulation and testing with Simulink Real-Time and Speedgoat hardware</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=xXNjLKcn0zE</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Real-Time Simulation and Testing I Webinar</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=P7Uy9RNwn8E</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Real-Time Simulation and Testing Part Four: Speedgoat for RCP and HIL</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=HUvNJd7UJnc</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>HIL Simulation and Testing with Simulink Real-Time and Speedgoat Target Hardware</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Rb3Aefnu0NY</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>HIL Simulation with Simulink &amp; Speedgoat</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=VBrY81ehiD0</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Introduction to Speedgoat FPGA Technology</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=WVHhhVgYnnI</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Enabling Innovation for Automotive HIL Testing and Control Design</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=5p_jsiEPRJE</t>
+        </is>
+      </c>
+    </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Speedgoat YouTube channel - all videos</t>
+          <t>Rapid Control Prototyping with Simulink Real-Time</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/c/SpeedgoatCh/videos</t>
+          <t>https://www.youtube.com/watch?v=45yv53-xX3w</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Rapid Control Prototyping for Power Electronics Control Design</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=WUXBXIY4Yc8</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Rapid Prototyping for Electric Motor Controls Design</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=_7XyCG9qS30</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Electric Motor Control | Rapid Control Prototyping, Part 2</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=RF2qioii_L0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Hardware-in-the-Loop Testing for Electric Motor Control</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=sESpcrn9BzU</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Power Electronics and Motor Control Prototyping on CPU/FPGA Target Hardware with Simulink Real-Time</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=KhqwoJITrMM</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Real-Time Simulation and Testing of PMSM Motors using Simulink Real-Time and Speedgoat</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=NSfh1FWAepA</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Hardware in the Loop Testing for Electric Powertrains</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Qgrz5jdWUeY</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>HIL Testing of Battery Management System (BMS)</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=AP0WEcZuxUg</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>HIL Testing of BMS using Simulink Real-Time and Speedgoat target hardware</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=FgkfSQ2Hk1k</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Motion Control Prototyping and PLC Testing in Automation Industry</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=PFbVTS71Duk</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Speedgoat Automotive Ad - Academic Institutions &amp; Corporates</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=rA3yHQPZG8c</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Speedgoat HiL and TPT - Set up the Execution Platform</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=zVp2jthmxv8</t>
         </is>
       </c>
     </row>
@@ -617,12 +925,186 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId23"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="80" customWidth="1" min="1" max="1"/>
+    <col width="115" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Real-Time Simulation and Testing: Hardware-in-the-Loop</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mathworks.com/videos/real-time-simulation-and-testing-hardware-in-the-loop-1597995453572.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Real-Time Simulation and Testing - Rapid Control Prototyping</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mathworks.com/videos/real-time-simulation-and-testing-rapid-control-prototyping-1600759638781.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>HIL Testing of Battery Management System (BMS) using Simulink Real-Time and Speedgoat target hardware</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mathworks.com/videos/hil-simulation-and-testing-with-simulink-real-time-and-speedgoat-target-hardware-116258.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>CPU, FPGA, and I/O Solutions for Real-Time Simulation and Testing with Simulink</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mathworks.com/videos/cpu-fpga-and-i-o-solutions-for-real-time-simulation-and-testing-with-simulink-1504019372112.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Introduction to Speedgoat FPGA Technology</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mathworks.com/videos/introduction-to-speedgoat-fpga-technology-1619157121683.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Full-switching Electric Drive FPGA-based Hardware-in-the-Loop Simulation</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mathworks.com/videos/full-switching-electric-drive-fpga-based-hardware-in-the-loop-simulation-1669999108325.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Nonlinear MPC Deployment to Speedgoat Hardware for Real-Time Testing (Understanding MPC, Part 9)</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mathworks.com/videos/understanding-model-predictive-control-part-9-nonlinear-mpc-deployment-to-speedgoat-hardware-for-real-time-testing-1659680359108.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Reinforcement Learning Agent Deployment: Real-Time Testing on a Speedgoat Machine</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mathworks.com/videos/reinforcement-learning-agent-deployment-real-time-testing-on-a-speedgoat-machine-1638925352260.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>From Modeling to Real-Time Prototyping with Speedgoat Hardware (German)</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mathworks.com/videos/from-modeling-to-real-time-prototyping-with-speedgoat-hardware-1599729325518.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Build and Run a Real-Time Application (Simulink Real-Time Explorer)</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mathworks.com/videos/simulink-real-time-explorer-1599736784381.html</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -631,7 +1113,7 @@
   <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="72" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="1" max="1"/>
     <col width="115" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -643,7 +1125,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Speedgoat URL</t>
+          <t>URL</t>
         </is>
       </c>
     </row>
@@ -758,16 +1240,16 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="130" customWidth="1" min="1" max="1"/>
+    <col width="135" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -780,35 +1262,42 @@
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>Collected 2026-07-20. speedgoat.com blocks automated crawling from this environment (HTTP 403 on direct requests, fetchers, and sitemap.xml), so URLs were gathered via search-engine indexes restricted to the speedgoat.com domain.</t>
+          <t>Collected 2026-07-20. speedgoat.com, youtube.com, and web.archive.org all block automated access from this environment, so every tab was built from search-engine indexes (domain-restricted queries), not a live crawl.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>Tab 1 'Video URLs' lists every discovered URL containing the word 'video' (10 speedgoat URLs + the Speedgoat YouTube channel).</t>
+          <t>Tab 1: every discovered speedgoat.com URL containing the word 'video'.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="5" t="inlineStr">
         <is>
-          <t>Tab 2 lists pages that host videos (tutorial series, learning videos) but whose URL does not contain the word 'video'.</t>
+          <t>Tab 2: Speedgoat's own YouTube channel (@SpeedgoatRT) and all of its videos found in search indexes (~20). The channel itself hosts the complete, authoritative set - open https://www.youtube.com/@SpeedgoatRT/videos in a browser to see every video.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>The Simulink Real-Time tutorial series is 5 parts per release (R2020a and R2020b); only the parts indexed by search engines are listed. The remaining parts likely exist at the same URL pattern (e.g. .../r2020b-slrt-part-2).</t>
+          <t>Tab 3: Speedgoat-related videos hosted on mathworks.com/videos (their partner MathWorks).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>This is broad coverage of indexed pages, not a guaranteed-complete crawl - pages not indexed by search engines cannot be discovered while the site blocks crawlers.</t>
+          <t>Tab 4: speedgoat.com pages that host videos but whose URL does not contain the word 'video' (tutorial series, learning videos).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Completeness: search indexes only surface videos that have been crawled and ranked; low-view or new videos may be missing. For a guaranteed-complete list, the two places to check in a normal browser are: (1) https://www.youtube.com/@SpeedgoatRT/videos and (2) https://www.speedgoat.com/knowledge-center filtered by Videos.</t>
         </is>
       </c>
     </row>

</xml_diff>